<commit_message>
Have conditional formatting on ambient illumination check monitor type
</commit_message>
<xml_diff>
--- a/MUSCMammoMonitor.xlsx
+++ b/MUSCMammoMonitor.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\workspace\EquipTestingSpreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CB544F-0450-48A3-9DC2-21A0B29942A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4B9A37-9CAF-4196-8B75-1ADED93BA4F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">BarcoYearlyChecks!$B$1:$L$46</definedName>
     <definedName name="Z_B8088769_C3DE_4DF8_A82B_D0EB46FFCC4A_.wvu.PrintArea" localSheetId="0" hidden="1">Barco!$B$1:$M$132</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateCount="1"/>
   <customWorkbookViews>
     <customWorkbookView name="Eugene Mah - Personal View" guid="{B8088769-C3DE-4DF8-A82B-D0EB46FFCC4A}" mergeInterval="0" personalView="1" maximized="1" xWindow="-8" yWindow="-8" windowWidth="1382" windowHeight="784" tabRatio="500" activeSheetId="1"/>
   </customWorkbookViews>
@@ -733,10 +733,10 @@
     <t>MDNG-6221</t>
   </si>
   <si>
-    <t>Revision 1.7-20250603</t>
-  </si>
-  <si>
     <t>MDNC-12130</t>
+  </si>
+  <si>
+    <t>Revision 1.7.1-20260409</t>
   </si>
 </sst>
 </file>
@@ -2330,6 +2330,72 @@
     <xf numFmtId="167" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2363,85 +2429,19 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2455,7 +2455,157 @@
     <cellStyle name="Result" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
     <cellStyle name="Result2" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="30">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2981,7 +3131,7 @@
       <c r="L1" s="3"/>
       <c r="M1" s="4"/>
       <c r="O1" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P1" s="6"/>
       <c r="Q1" s="6"/>
@@ -2996,12 +3146,12 @@
       <c r="AA1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="AG1" s="218" t="s">
+      <c r="AG1" s="191" t="s">
         <v>1</v>
       </c>
-      <c r="AH1" s="218"/>
-      <c r="AI1" s="218"/>
-      <c r="AJ1" s="218"/>
+      <c r="AH1" s="191"/>
+      <c r="AI1" s="191"/>
+      <c r="AJ1" s="191"/>
     </row>
     <row r="2" spans="1:36" ht="14.4" customHeight="1">
       <c r="A2" s="1">
@@ -3020,14 +3170,14 @@
       <c r="AA2" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="AG2" s="219" t="s">
+      <c r="AG2" s="192" t="s">
         <v>3</v>
       </c>
-      <c r="AH2" s="219"/>
-      <c r="AI2" s="220" t="s">
+      <c r="AH2" s="192"/>
+      <c r="AI2" s="193" t="s">
         <v>4</v>
       </c>
-      <c r="AJ2" s="220"/>
+      <c r="AJ2" s="193"/>
     </row>
     <row r="3" spans="1:36" ht="14.4" customHeight="1">
       <c r="A3" s="1">
@@ -3300,10 +3450,10 @@
         <v>Eugene Mah</v>
       </c>
       <c r="AF9"/>
-      <c r="AG9" s="222" t="s">
+      <c r="AG9" s="195" t="s">
         <v>201</v>
       </c>
-      <c r="AH9" s="223"/>
+      <c r="AH9" s="196"/>
     </row>
     <row r="10" spans="1:36" ht="14.4" customHeight="1">
       <c r="A10" s="1">
@@ -3313,19 +3463,19 @@
       <c r="D10" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="221" t="str">
+      <c r="E10" s="194" t="str">
         <f t="shared" ref="E10:E15" si="1">IF(R10="","",R10)</f>
         <v/>
       </c>
-      <c r="F10" s="221"/>
+      <c r="F10" s="194"/>
       <c r="I10" s="48" t="s">
         <v>32</v>
       </c>
-      <c r="J10" s="221" t="str">
+      <c r="J10" s="194" t="str">
         <f t="shared" ref="J10:J15" si="2">IF(V10="","",V10)</f>
         <v/>
       </c>
-      <c r="K10" s="221"/>
+      <c r="K10" s="194"/>
       <c r="M10" s="11"/>
       <c r="O10" s="12"/>
       <c r="Q10" s="20" t="s">
@@ -3373,19 +3523,19 @@
       <c r="D11" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="214" t="str">
+      <c r="E11" s="197" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F11" s="214"/>
+      <c r="F11" s="197"/>
       <c r="I11" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="J11" s="217" t="str">
+      <c r="J11" s="198" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K11" s="217"/>
+      <c r="K11" s="198"/>
       <c r="M11" s="11"/>
       <c r="O11" s="12"/>
       <c r="Q11" s="20" t="s">
@@ -3433,19 +3583,19 @@
       <c r="D12" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="214" t="str">
+      <c r="E12" s="197" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F12" s="214"/>
+      <c r="F12" s="197"/>
       <c r="I12" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="J12" s="214" t="str">
+      <c r="J12" s="197" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K12" s="214"/>
+      <c r="K12" s="197"/>
       <c r="M12" s="11"/>
       <c r="O12" s="12"/>
       <c r="Q12" s="20" t="s">
@@ -3460,7 +3610,7 @@
         <v>36</v>
       </c>
       <c r="V12" s="50" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(W12&lt;&gt;"",W12,IF(AB18="","",AB18))</f>
         <v/>
       </c>
       <c r="W12" s="51"/>
@@ -3493,19 +3643,19 @@
       <c r="D13" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="214" t="str">
+      <c r="E13" s="197" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F13" s="214"/>
+      <c r="F13" s="197"/>
       <c r="I13" s="48" t="s">
         <v>199</v>
       </c>
-      <c r="J13" s="214" t="str">
+      <c r="J13" s="197" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K13" s="214"/>
+      <c r="K13" s="197"/>
       <c r="M13" s="11"/>
       <c r="O13" s="12"/>
       <c r="Q13" s="20" t="s">
@@ -3520,7 +3670,7 @@
         <v>199</v>
       </c>
       <c r="V13" s="55" t="str">
-        <f t="shared" si="4"/>
+        <f>IF(W13&lt;&gt;"",W13,IF(AB19="","",AB19))</f>
         <v/>
       </c>
       <c r="W13" s="32"/>
@@ -3553,19 +3703,19 @@
       <c r="D14" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="214" t="str">
+      <c r="E14" s="197" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="F14" s="214"/>
+      <c r="F14" s="197"/>
       <c r="I14" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="J14" s="214" t="str">
+      <c r="J14" s="197" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K14" s="214"/>
+      <c r="K14" s="197"/>
       <c r="M14" s="11"/>
       <c r="O14" s="12"/>
       <c r="Q14" s="20" t="s">
@@ -3599,7 +3749,7 @@
       </c>
       <c r="AF14"/>
       <c r="AG14" s="15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="AH14" s="16">
         <v>40</v>
@@ -3613,19 +3763,19 @@
       <c r="D15" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="214" t="str">
+      <c r="E15" s="197" t="str">
         <f t="shared" si="1"/>
         <v>Barco K5905277 v18</v>
       </c>
-      <c r="F15" s="214"/>
+      <c r="F15" s="197"/>
       <c r="I15" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="J15" s="214" t="str">
+      <c r="J15" s="197" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="K15" s="214"/>
+      <c r="K15" s="197"/>
       <c r="M15" s="11"/>
       <c r="O15" s="25"/>
       <c r="P15" s="26"/>
@@ -3784,10 +3934,10 @@
       <c r="H19" s="136"/>
       <c r="I19" s="136"/>
       <c r="J19" s="136"/>
-      <c r="K19" s="216" t="s">
+      <c r="K19" s="200" t="s">
         <v>127</v>
       </c>
-      <c r="L19" s="216"/>
+      <c r="L19" s="200"/>
       <c r="M19" s="4"/>
       <c r="O19" s="12"/>
       <c r="R19" s="1" t="s">
@@ -4032,11 +4182,11 @@
       <c r="D24" s="48" t="s">
         <v>83</v>
       </c>
-      <c r="E24" s="215" t="str">
+      <c r="E24" s="199" t="str">
         <f>IF(P52="","",P52)</f>
         <v/>
       </c>
-      <c r="F24" s="215"/>
+      <c r="F24" s="199"/>
       <c r="M24" s="11"/>
       <c r="O24" s="12"/>
       <c r="Y24" s="13"/>
@@ -5896,16 +6046,16 @@
       </c>
       <c r="B71" s="9"/>
       <c r="C71" s="83"/>
-      <c r="D71" s="211" t="str">
+      <c r="D71" s="201" t="str">
         <f>Q86</f>
         <v>UNL-10 (cd/m^2)</v>
       </c>
-      <c r="E71" s="211"/>
-      <c r="F71" s="212" t="str">
+      <c r="E71" s="201"/>
+      <c r="F71" s="202" t="str">
         <f>S86</f>
         <v>UNL-80 (cd/m^2)</v>
       </c>
-      <c r="G71" s="212"/>
+      <c r="G71" s="202"/>
       <c r="I71" s="60" t="s">
         <v>106</v>
       </c>
@@ -6008,13 +6158,13 @@
       <c r="Q73" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="R73" s="194"/>
-      <c r="S73" s="198"/>
-      <c r="V73" s="206" t="str">
+      <c r="R73" s="216"/>
+      <c r="S73" s="220"/>
+      <c r="V73" s="208" t="str">
         <f>IF(AB48="","",AB48)</f>
         <v/>
       </c>
-      <c r="W73" s="207" t="str">
+      <c r="W73" s="209" t="str">
         <f>IF(AB51="","",AB51)</f>
         <v/>
       </c>
@@ -6056,10 +6206,10 @@
       <c r="M74" s="11"/>
       <c r="O74" s="12"/>
       <c r="Q74" s="19"/>
-      <c r="R74" s="195"/>
-      <c r="S74" s="199"/>
-      <c r="V74" s="205"/>
-      <c r="W74" s="208"/>
+      <c r="R74" s="217"/>
+      <c r="S74" s="221"/>
+      <c r="V74" s="207"/>
+      <c r="W74" s="210"/>
       <c r="Y74" s="13"/>
       <c r="AB74" s="139"/>
       <c r="AC74" s="34" t="str">
@@ -6100,13 +6250,13 @@
       <c r="Q75" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="R75" s="196"/>
-      <c r="S75" s="200"/>
-      <c r="V75" s="203" t="str">
+      <c r="R75" s="218"/>
+      <c r="S75" s="222"/>
+      <c r="V75" s="205" t="str">
         <f>IF(AB49="","",AB49)</f>
         <v/>
       </c>
-      <c r="W75" s="209" t="str">
+      <c r="W75" s="211" t="str">
         <f>IF(AB52="","",AB52)</f>
         <v/>
       </c>
@@ -6147,10 +6297,10 @@
       <c r="M76" s="11"/>
       <c r="O76" s="12"/>
       <c r="Q76" s="19"/>
-      <c r="R76" s="195"/>
-      <c r="S76" s="199"/>
-      <c r="V76" s="205"/>
-      <c r="W76" s="208"/>
+      <c r="R76" s="217"/>
+      <c r="S76" s="221"/>
+      <c r="V76" s="207"/>
+      <c r="W76" s="210"/>
       <c r="Y76" s="13"/>
       <c r="AB76" s="139"/>
       <c r="AC76" s="34" t="str">
@@ -6191,13 +6341,13 @@
       <c r="Q77" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="R77" s="196"/>
-      <c r="S77" s="200"/>
-      <c r="V77" s="203" t="str">
+      <c r="R77" s="218"/>
+      <c r="S77" s="222"/>
+      <c r="V77" s="205" t="str">
         <f>IF(AB50="","",AB50)</f>
         <v/>
       </c>
-      <c r="W77" s="209" t="str">
+      <c r="W77" s="211" t="str">
         <f>IF(AB53="","",AB53)</f>
         <v/>
       </c>
@@ -6213,10 +6363,10 @@
       <c r="M78" s="11"/>
       <c r="O78" s="12"/>
       <c r="Q78" s="19"/>
-      <c r="R78" s="197"/>
-      <c r="S78" s="201"/>
-      <c r="V78" s="204"/>
-      <c r="W78" s="210"/>
+      <c r="R78" s="219"/>
+      <c r="S78" s="223"/>
+      <c r="V78" s="206"/>
+      <c r="W78" s="212"/>
       <c r="Y78" s="13"/>
       <c r="AB78" s="139"/>
       <c r="AC78" s="34" t="str">
@@ -6403,16 +6553,16 @@
         <f>S68</f>
         <v>Right ()</v>
       </c>
-      <c r="I84" s="213" t="str">
+      <c r="I84" s="203" t="str">
         <f>R68</f>
         <v>Left ()</v>
       </c>
-      <c r="J84" s="213"/>
-      <c r="K84" s="213" t="str">
+      <c r="J84" s="203"/>
+      <c r="K84" s="203" t="str">
         <f>S68</f>
         <v>Right ()</v>
       </c>
-      <c r="L84" s="213"/>
+      <c r="L84" s="203"/>
       <c r="M84" s="11"/>
       <c r="O84" s="12"/>
       <c r="Y84" s="13"/>
@@ -6445,16 +6595,16 @@
       <c r="H85" s="48" t="s">
         <v>95</v>
       </c>
-      <c r="I85" s="202" t="str">
+      <c r="I85" s="204" t="str">
         <f>IF(R73="","",R73)</f>
         <v/>
       </c>
-      <c r="J85" s="202"/>
-      <c r="K85" s="202" t="str">
+      <c r="J85" s="204"/>
+      <c r="K85" s="204" t="str">
         <f>IF(S73="","",S73)</f>
         <v/>
       </c>
-      <c r="L85" s="202"/>
+      <c r="L85" s="204"/>
       <c r="M85" s="11"/>
       <c r="O85" s="97" t="s">
         <v>105</v>
@@ -6483,26 +6633,26 @@
       <c r="H86" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="I86" s="202" t="str">
+      <c r="I86" s="204" t="str">
         <f>IF(R75="","",R75)</f>
         <v/>
       </c>
-      <c r="J86" s="202"/>
-      <c r="K86" s="202" t="str">
+      <c r="J86" s="204"/>
+      <c r="K86" s="204" t="str">
         <f>IF(S75="","",S75)</f>
         <v/>
       </c>
-      <c r="L86" s="202"/>
+      <c r="L86" s="204"/>
       <c r="M86" s="11"/>
       <c r="O86" s="12"/>
-      <c r="Q86" s="192" t="s">
+      <c r="Q86" s="214" t="s">
         <v>116</v>
       </c>
-      <c r="R86" s="193"/>
-      <c r="S86" s="192" t="s">
+      <c r="R86" s="215"/>
+      <c r="S86" s="214" t="s">
         <v>117</v>
       </c>
-      <c r="T86" s="193"/>
+      <c r="T86" s="215"/>
       <c r="V86" s="113" t="s">
         <v>43</v>
       </c>
@@ -6527,16 +6677,16 @@
       <c r="H87" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="I87" s="191" t="str">
+      <c r="I87" s="213" t="str">
         <f>IF(R77="","",R77)</f>
         <v/>
       </c>
-      <c r="J87" s="191"/>
-      <c r="K87" s="191" t="str">
+      <c r="J87" s="213"/>
+      <c r="K87" s="213" t="str">
         <f>IF(S77="","",S77)</f>
         <v/>
       </c>
-      <c r="L87" s="191"/>
+      <c r="L87" s="213"/>
       <c r="M87" s="11"/>
       <c r="O87" s="12"/>
       <c r="Q87" s="114" t="str">
@@ -8243,36 +8393,6 @@
     </customSheetView>
   </customSheetViews>
   <mergeCells count="42">
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AG2:AH2"/>
-    <mergeCell ref="AI2:AJ2"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="AG9:AH9"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="I84:J84"/>
-    <mergeCell ref="K84:L84"/>
-    <mergeCell ref="I85:J85"/>
-    <mergeCell ref="K85:L85"/>
-    <mergeCell ref="V77:V78"/>
-    <mergeCell ref="V75:V76"/>
-    <mergeCell ref="V73:V74"/>
-    <mergeCell ref="W73:W74"/>
-    <mergeCell ref="W75:W76"/>
-    <mergeCell ref="W77:W78"/>
     <mergeCell ref="I87:J87"/>
     <mergeCell ref="K87:L87"/>
     <mergeCell ref="Q86:R86"/>
@@ -8285,6 +8405,36 @@
     <mergeCell ref="S77:S78"/>
     <mergeCell ref="I86:J86"/>
     <mergeCell ref="K86:L86"/>
+    <mergeCell ref="V77:V78"/>
+    <mergeCell ref="V75:V76"/>
+    <mergeCell ref="V73:V74"/>
+    <mergeCell ref="W73:W74"/>
+    <mergeCell ref="W75:W76"/>
+    <mergeCell ref="W77:W78"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="I84:J84"/>
+    <mergeCell ref="K84:L84"/>
+    <mergeCell ref="I85:J85"/>
+    <mergeCell ref="K85:L85"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AG2:AH2"/>
+    <mergeCell ref="AI2:AJ2"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="AG9:AH9"/>
   </mergeCells>
   <conditionalFormatting sqref="D27:D28">
     <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
@@ -8338,7 +8488,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="P26">
     <cfRule type="cellIs" dxfId="2" priority="16" operator="greaterThan">
-      <formula>20</formula>
+      <formula>VLOOKUP(V13,AG10:AH16,2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q99:T100">
@@ -8351,6 +8501,11 @@
       <formula>"VLOOKUP(V13,AG10:AH16,2)"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W13" xr:uid="{2CB91FFE-0AEC-45DD-ABF0-2B85C1E650EA}">
+      <formula1>$AG$11:$AG$16</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.78740157480314965" bottom="0.94488188976377963" header="0.51181102362204722" footer="0.78740157480314965"/>
   <pageSetup scale="65" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <headerFooter>
@@ -8493,19 +8648,19 @@
       <c r="D10" s="48" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="221" t="str">
+      <c r="E10" s="194" t="str">
         <f>Barco!E10</f>
         <v/>
       </c>
-      <c r="F10" s="221"/>
+      <c r="F10" s="194"/>
       <c r="I10" s="48" t="s">
         <v>32</v>
       </c>
-      <c r="J10" s="221" t="str">
+      <c r="J10" s="194" t="str">
         <f>Barco!J10</f>
         <v/>
       </c>
-      <c r="K10" s="221"/>
+      <c r="K10" s="194"/>
       <c r="L10" s="178"/>
     </row>
     <row r="11" spans="1:18">
@@ -8516,19 +8671,19 @@
       <c r="D11" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="221" t="str">
+      <c r="E11" s="194" t="str">
         <f>Barco!E11</f>
         <v/>
       </c>
-      <c r="F11" s="221"/>
+      <c r="F11" s="194"/>
       <c r="I11" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="J11" s="221" t="str">
+      <c r="J11" s="194" t="str">
         <f>Barco!J11</f>
         <v/>
       </c>
-      <c r="K11" s="221"/>
+      <c r="K11" s="194"/>
       <c r="L11" s="178"/>
     </row>
     <row r="12" spans="1:18">
@@ -8539,19 +8694,19 @@
       <c r="D12" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="221" t="str">
+      <c r="E12" s="194" t="str">
         <f>Barco!E12</f>
         <v/>
       </c>
-      <c r="F12" s="221"/>
+      <c r="F12" s="194"/>
       <c r="I12" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="J12" s="221" t="str">
+      <c r="J12" s="194" t="str">
         <f>Barco!J12</f>
         <v/>
       </c>
-      <c r="K12" s="221"/>
+      <c r="K12" s="194"/>
       <c r="L12" s="178"/>
     </row>
     <row r="13" spans="1:18">
@@ -8562,19 +8717,19 @@
       <c r="D13" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="E13" s="221" t="str">
+      <c r="E13" s="194" t="str">
         <f>Barco!E13</f>
         <v/>
       </c>
-      <c r="F13" s="221"/>
+      <c r="F13" s="194"/>
       <c r="I13" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="J13" s="221" t="str">
+      <c r="J13" s="194" t="str">
         <f>Barco!J14</f>
         <v/>
       </c>
-      <c r="K13" s="221"/>
+      <c r="K13" s="194"/>
       <c r="L13" s="178"/>
     </row>
     <row r="14" spans="1:18">
@@ -8585,19 +8740,19 @@
       <c r="D14" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="221" t="str">
+      <c r="E14" s="194" t="str">
         <f>Barco!E14</f>
         <v/>
       </c>
-      <c r="F14" s="221"/>
+      <c r="F14" s="194"/>
       <c r="I14" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="J14" s="221" t="str">
+      <c r="J14" s="194" t="str">
         <f>Barco!J15</f>
         <v/>
       </c>
-      <c r="K14" s="221"/>
+      <c r="K14" s="194"/>
       <c r="L14" s="178"/>
     </row>
     <row r="15" spans="1:18">
@@ -8608,11 +8763,11 @@
       <c r="D15" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="221" t="str">
+      <c r="E15" s="194" t="str">
         <f>Barco!E15</f>
         <v>Barco K5905277 v18</v>
       </c>
-      <c r="F15" s="221"/>
+      <c r="F15" s="194"/>
       <c r="L15" s="178"/>
     </row>
     <row r="16" spans="1:18" ht="16.2" thickBot="1">
@@ -8666,14 +8821,14 @@
         <v>20</v>
       </c>
       <c r="B20" s="177"/>
-      <c r="F20" s="228" t="s">
+      <c r="F20" s="224" t="s">
         <v>192</v>
       </c>
-      <c r="G20" s="228"/>
-      <c r="H20" s="228" t="s">
+      <c r="G20" s="224"/>
+      <c r="H20" s="224" t="s">
         <v>193</v>
       </c>
-      <c r="I20" s="228"/>
+      <c r="I20" s="224"/>
       <c r="L20" s="178"/>
     </row>
     <row r="21" spans="1:12">
@@ -8681,16 +8836,16 @@
         <v>21</v>
       </c>
       <c r="B21" s="177"/>
-      <c r="F21" s="228" t="str">
+      <c r="F21" s="224" t="str">
         <f>J13</f>
         <v/>
       </c>
-      <c r="G21" s="228"/>
-      <c r="H21" s="228" t="str">
+      <c r="G21" s="224"/>
+      <c r="H21" s="224" t="str">
         <f>J14</f>
         <v/>
       </c>
-      <c r="I21" s="228"/>
+      <c r="I21" s="224"/>
       <c r="L21" s="178"/>
     </row>
     <row r="22" spans="1:12">
@@ -8701,13 +8856,13 @@
       <c r="E22" s="48" t="s">
         <v>185</v>
       </c>
-      <c r="F22" s="227" t="str">
+      <c r="F22" s="226" t="str">
         <f>IF(Barco!E23="","",IF(Barco!E23="YES","PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="G22" s="227"/>
-      <c r="H22" s="227"/>
-      <c r="I22" s="227"/>
+      <c r="G22" s="226"/>
+      <c r="H22" s="226"/>
+      <c r="I22" s="226"/>
       <c r="L22" s="178"/>
     </row>
     <row r="23" spans="1:12">
@@ -8718,13 +8873,13 @@
       <c r="E23" s="48" t="s">
         <v>186</v>
       </c>
-      <c r="F23" s="227" t="str">
+      <c r="F23" s="226" t="str">
         <f>IF(Barco!E22="","",IF(Barco!E22="YES","PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="G23" s="227"/>
-      <c r="H23" s="227"/>
-      <c r="I23" s="227"/>
+      <c r="G23" s="226"/>
+      <c r="H23" s="226"/>
+      <c r="I23" s="226"/>
       <c r="L23" s="178"/>
     </row>
     <row r="24" spans="1:12">
@@ -8735,13 +8890,13 @@
       <c r="E24" s="48" t="s">
         <v>187</v>
       </c>
-      <c r="F24" s="227" t="str">
+      <c r="F24" s="226" t="str">
         <f>IF(OR(Barco!I72="TBD",Barco!I73="TBD"),"",IF(AND(Barco!I72="YES",Barco!I73="YES"),"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="G24" s="227"/>
-      <c r="H24" s="227"/>
-      <c r="I24" s="227"/>
+      <c r="G24" s="226"/>
+      <c r="H24" s="226"/>
+      <c r="I24" s="226"/>
       <c r="L24" s="178"/>
     </row>
     <row r="25" spans="1:12">
@@ -8752,10 +8907,10 @@
       <c r="E25" s="48" t="s">
         <v>188</v>
       </c>
-      <c r="F25" s="224"/>
-      <c r="G25" s="224"/>
-      <c r="H25" s="224"/>
-      <c r="I25" s="224"/>
+      <c r="F25" s="225"/>
+      <c r="G25" s="225"/>
+      <c r="H25" s="225"/>
+      <c r="I25" s="225"/>
       <c r="L25" s="178"/>
     </row>
     <row r="26" spans="1:12">
@@ -8769,13 +8924,13 @@
       <c r="E26" s="48" t="s">
         <v>189</v>
       </c>
-      <c r="F26" s="227" t="str">
+      <c r="F26" s="226" t="str">
         <f>IF(Barco!F85="","",IF(Barco!F85="YES","PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="G26" s="227"/>
-      <c r="H26" s="227"/>
-      <c r="I26" s="227"/>
+      <c r="G26" s="226"/>
+      <c r="H26" s="226"/>
+      <c r="I26" s="226"/>
       <c r="L26" s="178"/>
     </row>
     <row r="27" spans="1:12">
@@ -8786,10 +8941,10 @@
       <c r="E27" s="48" t="s">
         <v>190</v>
       </c>
-      <c r="F27" s="224"/>
-      <c r="G27" s="224"/>
-      <c r="H27" s="224"/>
-      <c r="I27" s="224"/>
+      <c r="F27" s="225"/>
+      <c r="G27" s="225"/>
+      <c r="H27" s="225"/>
+      <c r="I27" s="225"/>
       <c r="L27" s="178"/>
     </row>
     <row r="28" spans="1:12">
@@ -8800,10 +8955,10 @@
       <c r="E28" s="48" t="s">
         <v>191</v>
       </c>
-      <c r="F28" s="224"/>
-      <c r="G28" s="224"/>
-      <c r="H28" s="224"/>
-      <c r="I28" s="224"/>
+      <c r="F28" s="225"/>
+      <c r="G28" s="225"/>
+      <c r="H28" s="225"/>
+      <c r="I28" s="225"/>
       <c r="L28" s="178"/>
     </row>
     <row r="29" spans="1:12">
@@ -8814,16 +8969,16 @@
       <c r="E29" s="48" t="s">
         <v>197</v>
       </c>
-      <c r="F29" s="225" t="str">
+      <c r="F29" s="227" t="str">
         <f>IF(Barco!F86="","",IF(Barco!F86="YES","PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="G29" s="226"/>
-      <c r="H29" s="225" t="str">
+      <c r="G29" s="228"/>
+      <c r="H29" s="227" t="str">
         <f>IF(Barco!G86="","",IF(Barco!G86="YES","PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="I29" s="226"/>
+      <c r="I29" s="228"/>
       <c r="L29" s="178"/>
     </row>
     <row r="30" spans="1:12">
@@ -8997,12 +9152,15 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H26:I26"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="E13:F13"/>
@@ -9019,15 +9177,12 @@
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H22:I22"/>
     <mergeCell ref="H23:I23"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="J12:K12"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F25:I25 F27:I28" xr:uid="{CEAD9B4F-4A05-4883-9435-EBBC3722EE42}">

</xml_diff>

<commit_message>
Lookup list for test equipment
</commit_message>
<xml_diff>
--- a/MUSCMammoMonitor.xlsx
+++ b/MUSCMammoMonitor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\workspace\EquipTestingSpreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4B9A37-9CAF-4196-8B75-1ADED93BA4F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7022693-C4B7-493F-8A24-DD69E0F7DE94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="216">
   <si>
     <t>Print Area</t>
   </si>
@@ -737,6 +737,21 @@
   </si>
   <si>
     <t>Revision 1.7.1-20260409</t>
+  </si>
+  <si>
+    <t>RTI Piranha</t>
+  </si>
+  <si>
+    <t>Piranha 1</t>
+  </si>
+  <si>
+    <t>Piranha 1 CB2-17090320</t>
+  </si>
+  <si>
+    <t>Piranha 2</t>
+  </si>
+  <si>
+    <t>Piranha 2 CB2-19020491</t>
   </si>
 </sst>
 </file>
@@ -1762,7 +1777,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="230">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2444,6 +2459,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Fail" xfId="6" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -3856,7 +3872,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:33" ht="14.4" customHeight="1" thickTop="1" thickBot="1">
+    <row r="17" spans="1:34" ht="14.4" customHeight="1" thickTop="1" thickBot="1">
       <c r="A17" s="1">
         <v>17</v>
       </c>
@@ -3883,7 +3899,7 @@
       <c r="AF17"/>
       <c r="AG17"/>
     </row>
-    <row r="18" spans="1:33" ht="14.4" customHeight="1" thickBot="1">
+    <row r="18" spans="1:34" ht="14.4" customHeight="1" thickBot="1">
       <c r="A18" s="1">
         <v>18</v>
       </c>
@@ -3917,9 +3933,11 @@
         <v/>
       </c>
       <c r="AF18"/>
-      <c r="AG18"/>
-    </row>
-    <row r="19" spans="1:33" ht="14.4" customHeight="1" thickTop="1">
+      <c r="AG18" s="229" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="19" spans="1:34" ht="14.4" customHeight="1" thickTop="1">
       <c r="A19" s="1">
         <v>19</v>
       </c>
@@ -3960,9 +3978,14 @@
         <v/>
       </c>
       <c r="AF19"/>
-      <c r="AG19"/>
-    </row>
-    <row r="20" spans="1:33" ht="14.4" customHeight="1">
+      <c r="AG19" s="229" t="s">
+        <v>212</v>
+      </c>
+      <c r="AH19" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:34" ht="14.4" customHeight="1">
       <c r="A20" s="1">
         <v>20</v>
       </c>
@@ -4019,9 +4042,14 @@
         <v/>
       </c>
       <c r="AF20"/>
-      <c r="AG20"/>
-    </row>
-    <row r="21" spans="1:33" ht="14.4" customHeight="1">
+      <c r="AG20" s="229" t="s">
+        <v>214</v>
+      </c>
+      <c r="AH20" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="21" spans="1:34" ht="14.4" customHeight="1">
       <c r="A21" s="1">
         <v>21</v>
       </c>
@@ -4044,9 +4072,9 @@
       <c r="K21" s="48" t="s">
         <v>126</v>
       </c>
-      <c r="L21" s="185">
+      <c r="L21" s="185" t="str">
         <f t="shared" ref="L21:L22" si="8">IF(W21="","",W21)</f>
-        <v>45089</v>
+        <v/>
       </c>
       <c r="M21" s="11"/>
       <c r="O21" s="65"/>
@@ -4057,13 +4085,11 @@
       <c r="V21" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="W21" s="135">
+      <c r="W21" s="135" t="str">
         <f t="shared" ref="W21:W22" si="9">IF(X21&lt;&gt;"",X21,IF(AB24="","",AB24))</f>
-        <v>45089</v>
-      </c>
-      <c r="X21" s="187">
-        <v>45089</v>
-      </c>
+        <v/>
+      </c>
+      <c r="X21" s="187"/>
       <c r="Y21" s="13"/>
       <c r="AA21" s="20" t="s">
         <v>40</v>
@@ -4082,7 +4108,7 @@
       <c r="AF21"/>
       <c r="AG21"/>
     </row>
-    <row r="22" spans="1:33" ht="14.4" customHeight="1">
+    <row r="22" spans="1:34" ht="14.4" customHeight="1">
       <c r="A22" s="1">
         <v>22</v>
       </c>
@@ -4105,9 +4131,9 @@
       <c r="K22" s="48" t="s">
         <v>125</v>
       </c>
-      <c r="L22" s="185">
+      <c r="L22" s="185" t="str">
         <f t="shared" si="8"/>
-        <v>45820</v>
+        <v/>
       </c>
       <c r="M22" s="11"/>
       <c r="O22" s="65"/>
@@ -4118,13 +4144,11 @@
       <c r="V22" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="W22" s="135">
+      <c r="W22" s="135" t="str">
         <f t="shared" si="9"/>
-        <v>45820</v>
-      </c>
-      <c r="X22" s="187">
-        <v>45820</v>
-      </c>
+        <v/>
+      </c>
+      <c r="X22" s="187"/>
       <c r="Y22" s="13"/>
       <c r="AA22" s="20" t="s">
         <v>127</v>
@@ -4132,7 +4156,7 @@
       <c r="AF22"/>
       <c r="AG22"/>
     </row>
-    <row r="23" spans="1:33" ht="14.4" customHeight="1">
+    <row r="23" spans="1:34" ht="14.4" customHeight="1">
       <c r="A23" s="1">
         <v>23</v>
       </c>
@@ -4174,7 +4198,7 @@
       <c r="AF23"/>
       <c r="AG23"/>
     </row>
-    <row r="24" spans="1:33" ht="14.4" customHeight="1">
+    <row r="24" spans="1:34" ht="14.4" customHeight="1">
       <c r="A24" s="1">
         <v>24</v>
       </c>
@@ -4196,16 +4220,16 @@
       <c r="AB24" s="134"/>
       <c r="AC24" s="34" t="str">
         <f t="shared" si="10"/>
-        <v>Change</v>
-      </c>
-      <c r="AD24" s="133">
+        <v/>
+      </c>
+      <c r="AD24" s="133" t="str">
         <f t="shared" ref="AD24:AD25" si="11">IF(X21="","",X21)</f>
-        <v>45089</v>
+        <v/>
       </c>
       <c r="AF24"/>
       <c r="AG24"/>
     </row>
-    <row r="25" spans="1:33" ht="14.4" customHeight="1">
+    <row r="25" spans="1:34" ht="14.4" customHeight="1">
       <c r="A25" s="1">
         <v>25</v>
       </c>
@@ -4227,16 +4251,16 @@
       <c r="AB25" s="134"/>
       <c r="AC25" s="34" t="str">
         <f t="shared" si="10"/>
-        <v>Change</v>
-      </c>
-      <c r="AD25" s="133">
+        <v/>
+      </c>
+      <c r="AD25" s="133" t="str">
         <f t="shared" si="11"/>
-        <v>45820</v>
+        <v/>
       </c>
       <c r="AF25"/>
       <c r="AG25"/>
     </row>
-    <row r="26" spans="1:33" ht="14.4" customHeight="1">
+    <row r="26" spans="1:34" ht="14.4" customHeight="1">
       <c r="A26" s="1">
         <v>26</v>
       </c>
@@ -4266,7 +4290,7 @@
       <c r="AF26"/>
       <c r="AG26"/>
     </row>
-    <row r="27" spans="1:33" ht="14.4" customHeight="1">
+    <row r="27" spans="1:34" ht="14.4" customHeight="1">
       <c r="A27" s="1">
         <v>27</v>
       </c>
@@ -4325,7 +4349,7 @@
       <c r="AF27"/>
       <c r="AG27"/>
     </row>
-    <row r="28" spans="1:33" ht="14.4" customHeight="1">
+    <row r="28" spans="1:34" ht="14.4" customHeight="1">
       <c r="A28" s="1">
         <v>28</v>
       </c>
@@ -4365,7 +4389,7 @@
       <c r="AF28"/>
       <c r="AG28"/>
     </row>
-    <row r="29" spans="1:33" ht="14.4" customHeight="1">
+    <row r="29" spans="1:34" ht="14.4" customHeight="1">
       <c r="A29" s="1">
         <v>29</v>
       </c>
@@ -4415,7 +4439,7 @@
       <c r="AF29"/>
       <c r="AG29"/>
     </row>
-    <row r="30" spans="1:33" ht="14.4" customHeight="1">
+    <row r="30" spans="1:34" ht="14.4" customHeight="1">
       <c r="A30" s="1">
         <v>30</v>
       </c>
@@ -4464,7 +4488,7 @@
       <c r="AF30"/>
       <c r="AG30"/>
     </row>
-    <row r="31" spans="1:33" ht="14.4" customHeight="1">
+    <row r="31" spans="1:34" ht="14.4" customHeight="1">
       <c r="A31" s="1">
         <v>31</v>
       </c>
@@ -4510,7 +4534,7 @@
       <c r="AF31"/>
       <c r="AG31"/>
     </row>
-    <row r="32" spans="1:33" ht="14.4" customHeight="1">
+    <row r="32" spans="1:34" ht="14.4" customHeight="1">
       <c r="A32" s="1">
         <v>32</v>
       </c>
@@ -8501,9 +8525,12 @@
       <formula>"VLOOKUP(V13,AG10:AH16,2)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W13" xr:uid="{2CB91FFE-0AEC-45DD-ABF0-2B85C1E650EA}">
       <formula1>$AG$11:$AG$16</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X20" xr:uid="{5E493689-B45C-488F-8D1F-460E5B66E402}">
+      <formula1>$AH$19:$AH$20</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.78740157480314965" bottom="0.94488188976377963" header="0.51181102362204722" footer="0.78740157480314965"/>

</xml_diff>